<commit_message>
Éléments répétés : chaque semaine, mois, trimestre ou année
- Répétition à jour précis ou « dans la période », avec début et fin
- Cocher valide la période en cours ; l'élément revient à la suivante
- Périodes oubliées à rattraper, regroupées sur une ligne « En retard »
  (cocher valide la plus ancienne)
- Liste : sections Cette semaine / Ce mois-ci / Ce trimestre ; pas d'affichage en avance
- Vues Semaine et Mois : échéances dans le calendrier et bandeau « à faire sur la période »
- Filtre 🔁, badge de période, résumé « Chaque mois, le 5 » dans le formulaire
- Script : 5 colonnes ajoutées automatiquement à un onglet existant (sans perte),
  validation, version d'API ; l'application prévient si le script n'est pas à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -54,10 +54,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -437,6 +438,11 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,6 +501,31 @@
           <t>modifie_le</t>
         </is>
       </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>periodicite</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>echeance</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>debut</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>fin</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>faits</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -552,6 +583,11 @@
           <t>2026-09-23T13:00:00.000Z</t>
         </is>
       </c>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -601,6 +637,11 @@
           <t>2026-09-23T13:00:00.000Z</t>
         </is>
       </c>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
SAFe étape 3 : features, objectifs du PI, écran PI
- Features (sous-epics) : epic, PI, itération prévue, points, tâches ; suppression
  avec ou sans ses tâches (sinon elles remontent à l'epic)
- Objectifs du PI : engagé / bonus, valeur prévue et obtenue sur 10, prévisibilité
- Écran PI : objectifs du PI, tableau features × itérations groupé par epic
  (itération prévue, tâches faites / total par itération), charge par itération
  face à la capacité, features sans PI, navigation entre PI
- Menu + selon l'écran (feature, objectif du PI) ; features listées sous leur epic
  dans la roadmap en mode SAFe
- README et modèle Excel : nouveaux onglets et colonnes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Epics" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Objectifs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Domaines" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Features" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ObjectifsPI" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -449,6 +451,9 @@
     <col width="38" customWidth="1" min="17" max="17"/>
     <col width="38" customWidth="1" min="18" max="18"/>
     <col width="38" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="38" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -545,6 +550,21 @@
       <c r="S1" s="3" t="inlineStr">
         <is>
           <t>domaine</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>points</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t>iteration</t>
+        </is>
+      </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>feature</t>
         </is>
       </c>
     </row>
@@ -612,6 +632,9 @@
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -669,6 +692,9 @@
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="n"/>
       <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="n"/>
+      <c r="U3" s="2" t="n"/>
+      <c r="V3" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -681,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -694,6 +720,7 @@
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -745,6 +772,11 @@
       <c r="J1" s="3" t="inlineStr">
         <is>
           <t>domaine</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>etat</t>
         </is>
       </c>
     </row>
@@ -895,4 +927,148 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>titre</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>pi</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>iteration</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>points</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>couleur</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>cree_le</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>modifie_le</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>titre</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>pi</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>valeur_prevue</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>valeur_obtenue</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>cree_le</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>modifie_le</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Filtre de domaine partagé et objectifs du PI par domaine
- Filtre de domaine unique pour Tâches, Itération, PI, Roadmap et Portefeuille,
  mémorisé sur l'appareil ; capacité commune (charge du domaine + total / capacité,
  autres domaines en gris dans l'Itération)
- PI : objectifs, features, tâches hors feature et prévisibilité du domaine filtré
- Objectif du PI rattaché à un domaine (colonne domaine, script v6) ; supprimer un
  domaine ne supprime pas ses objectifs du PI, ils passent sans domaine
- Démo, modèle Excel et README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1024,6 +1024,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1065,6 +1066,11 @@
       <c r="H1" s="3" t="inlineStr">
         <is>
           <t>modifie_le</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>domaine</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nouveaux types : appel, démarche, story, exploration, bug
- 8 types identiques en mode Simple et SAFe, avec icône et couleur
- Appel : numéro de téléphone et bouton Appeler (fiche et liste)
- Filtre de la liste : Tous + liste déroulante des types (et répétés)
- Script v7 : nouveaux types acceptés, colonne telephone ajoutée sans perte ;
  l'application refuse d'enregistrer un nouveau type tant que le script n'est pas à jour
- Démo : exemples d'appel, démarche, story, exploration et bug ; modèle Excel et README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -565,6 +565,11 @@
       <c r="V1" s="3" t="inlineStr">
         <is>
           <t>feature</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>telephone</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rendez-vous : heure de fin, et alerte de chevauchement précise
- Script v9 : colonne heure_fin (après heure_fin > heure), ajoutée sans perte
- Fiche d'un rendez-vous : heure de fin (proposée 1 h après le début), durée
- Liste : « 🕒 10:30 → 11:30 »
- Alerte : créneaux qui se recouvrent réellement (sans fin : 1 h estimée), durée
  du chevauchement ou « a lieu pendant », bouton « Décaler … juste après »
- Démo, modèle Excel et README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -575,6 +575,11 @@
       <c r="X1" s="3" t="inlineStr">
         <is>
           <t>parent</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>heure_fin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alertes : ignorer (partagé via le Google Sheet) et corrections de règles
- Ignorer une alerte : enregistrée dans l'onglet Ignorees (script v10) avec la
  situation du moment ; elle revient si la situation change ; « les revoir » et
  « Ne plus ignorer » ; les ignorées ne comptent plus dans les onglets
- Agenda : chevauchements sur tout l'agenda malgré le filtre de domaine, rendez-vous
  répétés (30 jours), appels et missions avec une heure (30 min estimées)
- Rendez-vous passé : Marquer fait / Reprogrammer
- Retard d'une tâche et de ses sous-tâches regroupé ; parent « commencé » si une
  sous-tâche avance
- Pas d'alerte vide pour une epic Idée ou qui commence plus tard (idem objectif),
  ni délaissé pour un domaine récent
- Points parent ≠ sous-tâches : seulement dans l'Itération en mode SAFe

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Domaines" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Features" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="ObjectifsPI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Ignorees" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1092,4 +1093,52 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>cle</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>signature</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>cree_le</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>modifie_le</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Objectifs du PI : epic en plus du domaine, alerte « aucune feature ou tâche »
- Script v11 : colonne epic dans ObjectifsPI ; supprimer une epic la retire des
  objectifs du PI (qui gardent leur domaine)
- Fiche objectif du PI : choix de l'epic (range l'objectif dans son domaine)
- Alerte : engagé mais aucune feature ou tâche de son epic (sinon de son domaine)
  prévue dans le PI ; bouton « + Tâche dans l'epic »

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1041,6 +1041,7 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1087,6 +1088,11 @@
       <c r="I1" s="3" t="inlineStr">
         <is>
           <t>domaine</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>epic</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Démarches : date de fin ; alertes : 5 corrections, fin de l'alerte « 3 jours »
- Script v12 : colonne date_fin (date limite d'une démarche), affichée « ⏳ fin »
  dans la liste et prise en compte dans les alertes de dates de la roadmap
- Suppression de l'alerte « prévue dans 3 jours et pas commencée »
- Fin d'itération : sans les rendez-vous
- PI : « noter la valeur obtenue » aussi pour le PI qui vient de finir
- Roadmap : les alertes de dates des barres peuvent être ignorées
- Rendez-vous répétés : « n'est pas coché » / « Marquer fait » ; bon mot par type
- Domaine délaissé : rien de fait depuis 2 mois et rien de prévu

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:Z3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -455,6 +455,8 @@
     <col width="8" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="38" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -581,6 +583,11 @@
       <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>heure_fin</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>date_fin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Statuts : fiche alignée, parent qui suit ses sous-tâches, « terminé le », rdv/appel
- Fiche : « Terminé » d'un parent → terminer aussi les sous-tâches ? ; mémoire
  du statut d'avant mise à jour (fiche, boutons d'alertes)
- Parent : sous-tâche rouverte → parent Terminé repasse En cours ; sous-tâche
  commencée ou finie → parent À faire passe En cours (parentsLies)
- Script v13 : colonne termine_le (jour réel de fin), utilisée par le burndown
  et « domaine délaissé »
- Rendez-vous et appels : pas d'« En cours » (Kanban et fiche)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z3"/>
+  <dimension ref="A1:AA3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -457,6 +457,7 @@
     <col width="38" customWidth="1" min="22" max="22"/>
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -588,6 +589,11 @@
       <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>date_fin</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>termine_le</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Statuts : parent terminé avec sous-tâches ouvertes, statut d'avant dans le Sheet
- Alerte : tâche terminée alors que des sous-tâches ne sont pas faites (terminer
  aussi les sous-tâches / rouvrir) ; ces sous-tâches ne sont plus « en retard »
- Script v14 : colonne statut_avant (En cours avant Terminé), pour que décocher
  remette En cours sur tous les appareils

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LeQUBTNVMcA24UzJSpaoD
</commit_message>
<xml_diff>
--- a/modele/Taches.xlsx
+++ b/modele/Taches.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -458,6 +458,7 @@
     <col width="13" customWidth="1" min="25" max="25"/>
     <col width="13" customWidth="1" min="26" max="26"/>
     <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -594,6 +595,11 @@
       <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>termine_le</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>statut_avant</t>
         </is>
       </c>
     </row>

</xml_diff>